<commit_message>
machine learning with knapsack
</commit_message>
<xml_diff>
--- a/ml.xlsx
+++ b/ml.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,13 +489,18 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>BudgetImpact</t>
+          <t>QuantityToReduce</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ReducedBudgetImpact</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>5312</v>
+        <v>5294</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -504,25 +509,25 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ERASER, rubber</t>
+          <t>INK CART, EPSON L3110, Magenta 003</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>piece</t>
+          <t>bottle</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4.47</v>
+        <v>300</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -532,7 +537,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>COMMON OFFICE SUPPLIES</t>
+          <t>INK/TONER FOR PRINTER</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -541,18 +546,21 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>0.39</v>
+        <v>0.83</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O2" t="n">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2400</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>5417</v>
+        <v>5399</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -561,22 +569,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ERASER, rubber</t>
+          <t>INK CART, EPSON L3110, Magenta 003</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>piece</t>
+          <t>bottle</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4.47</v>
+        <v>300</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -589,7 +597,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>COMMON OFFICE SUPPLIES</t>
+          <t>INK/TONER FOR PRINTER</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -598,18 +606,21 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>0.39</v>
+        <v>0.83</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O3" t="n">
-        <v>22</v>
+        <v>9</v>
+      </c>
+      <c r="P3" t="n">
+        <v>2700</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5444</v>
+        <v>5400</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -618,22 +629,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RULER, plastic, 300mm, 1 piece in individual plastic (12")</t>
+          <t>INK CART, EPSON L3110, Yellow 003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>piece</t>
+          <t>bottle</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>16.64</v>
+        <v>300</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -646,7 +657,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>COMMON OFFICE SUPPLIES</t>
+          <t>INK/TONER FOR PRINTER</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -655,42 +666,45 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>0.39</v>
+        <v>0.83</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O4" t="n">
-        <v>33</v>
+        <v>9</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2700</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1088</v>
+        <v>5398</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-13T04:46:02.951308+00:00</t>
+          <t>2026-07-27T16:12:37.556591+00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ERASER rubber</t>
+          <t>INK CART, EPSON L3110, Cyan 003</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>piece</t>
+          <t>bottle</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4.47</v>
+        <v>300</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -699,54 +713,61 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>7</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
+        <v>32</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>INK/TONER FOR PRINTER</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Office Supply</t>
+          <t>Laboratory Supply/Equipment</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>0.38</v>
+        <v>0.83</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O5" t="n">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5700</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5507</v>
+        <v>5292</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-31T01:05:30.101366+00:00</t>
+          <t>2026-07-27T16:12:37.255204+00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>INK CART, EPSON L3110, Black 003</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>aaa</t>
+          <t>bottle</t>
         </is>
       </c>
       <c r="E6" t="n">
+        <v>300</v>
+      </c>
+      <c r="F6" t="n">
+        <v>25</v>
+      </c>
+      <c r="G6" t="n">
+        <v>24</v>
+      </c>
+      <c r="H6" t="n">
         <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -754,19 +775,322 @@
       <c r="J6" t="n">
         <v>32</v>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>INK/TONER FOR PRINTER</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>Office Supply</t>
         </is>
       </c>
       <c r="M6" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="N6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O6" t="n">
+        <v>24</v>
+      </c>
+      <c r="P6" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5397</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-27T16:12:37.556591+00:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>INK CART, EPSON L3110, Black 003</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>bottle</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>300</v>
+      </c>
+      <c r="F7" t="n">
+        <v>25</v>
+      </c>
+      <c r="G7" t="n">
+        <v>25</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>32</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>INK/TONER FOR PRINTER</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Laboratory Supply/Equipment</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="N7" t="n">
+        <v>18</v>
+      </c>
+      <c r="O7" t="n">
+        <v>21</v>
+      </c>
+      <c r="P7" t="n">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5296</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-27T16:12:37.255204+00:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Toner Cart, Copier Muratec MFX - 2835 with ADF</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>cartridge</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>32</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>INK/TONER FOR PHOTOCOPYING MACHINE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Office Supply</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>8</v>
+      </c>
+      <c r="P8" t="n">
+        <v>25600</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5401</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-27T16:12:37.556591+00:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Toner Cart, Copier Muratec MFX - 2835 with ADF</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>cartridge</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>32</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>INK/TONER FOR PHOTOCOPYING MACHINE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Laboratory Supply/Equipment</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2</v>
+      </c>
+      <c r="P9" t="n">
+        <v>6400</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5303</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-27T16:12:37.255204+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CLIP, backfold, 19mm, 12 pieces per box</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>box</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>32</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>COMMON OFFICE SUPPLIES</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Office Supply</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
         <v>0.38</v>
       </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>8.720000000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5507</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-31T01:05:30.101366+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>32</v>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Office Supply</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding item 0 in ml
</commit_message>
<xml_diff>
--- a/ml.xlsx
+++ b/ml.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,75 +424,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>ItemName</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ItemName</t>
+          <t>UnitName</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>UnitName</t>
+          <t>AI_Score</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>QuantityToReduce</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>PricePerUnit</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>PlannedQuantity</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>AvailableQuantity</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>PendingQuantity</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>FulfilledQuantity</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>FiscalYearID</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ItemCategory</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>PpmpCategory</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>AI_Score</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>InLieuTotalQuantity</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>QuantityToReduce</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
         <is>
           <t>ReducedBudgetImpact</t>
         </is>
@@ -504,57 +459,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.255204+00:00</t>
+          <t>INK CART, EPSON L3110, Magenta 003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>INK CART, EPSON L3110, Magenta 003</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
           <t>bottle</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>0.83</v>
+      </c>
       <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
         <v>300</v>
       </c>
-      <c r="F2" t="n">
-        <v>9</v>
-      </c>
       <c r="G2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>32</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PRINTER</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Office Supply</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="N2" t="n">
-        <v>18</v>
-      </c>
-      <c r="O2" t="n">
-        <v>8</v>
-      </c>
-      <c r="P2" t="n">
         <v>2400</v>
       </c>
     </row>
@@ -564,57 +486,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.556591+00:00</t>
+          <t>INK CART, EPSON L3110, Magenta 003</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>INK CART, EPSON L3110, Magenta 003</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
           <t>bottle</t>
         </is>
       </c>
+      <c r="D3" t="n">
+        <v>0.83</v>
+      </c>
       <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="n">
         <v>300</v>
       </c>
-      <c r="F3" t="n">
-        <v>9</v>
-      </c>
       <c r="G3" t="n">
-        <v>9</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>32</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PRINTER</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Laboratory Supply/Equipment</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="N3" t="n">
-        <v>18</v>
-      </c>
-      <c r="O3" t="n">
-        <v>9</v>
-      </c>
-      <c r="P3" t="n">
         <v>2700</v>
       </c>
     </row>
@@ -624,57 +513,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.556591+00:00</t>
+          <t>INK CART, EPSON L3110, Yellow 003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>INK CART, EPSON L3110, Yellow 003</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
           <t>bottle</t>
         </is>
       </c>
+      <c r="D4" t="n">
+        <v>0.83</v>
+      </c>
       <c r="E4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" t="n">
         <v>300</v>
       </c>
-      <c r="F4" t="n">
-        <v>9</v>
-      </c>
       <c r="G4" t="n">
-        <v>9</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>32</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PRINTER</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Laboratory Supply/Equipment</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="N4" t="n">
-        <v>18</v>
-      </c>
-      <c r="O4" t="n">
-        <v>9</v>
-      </c>
-      <c r="P4" t="n">
         <v>2700</v>
       </c>
     </row>
@@ -684,57 +540,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.556591+00:00</t>
+          <t>INK CART, EPSON L3110, Cyan 003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>INK CART, EPSON L3110, Cyan 003</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
           <t>bottle</t>
         </is>
       </c>
+      <c r="D5" t="n">
+        <v>0.83</v>
+      </c>
       <c r="E5" t="n">
+        <v>19</v>
+      </c>
+      <c r="F5" t="n">
         <v>300</v>
       </c>
-      <c r="F5" t="n">
-        <v>19</v>
-      </c>
       <c r="G5" t="n">
-        <v>19</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>32</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PRINTER</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Laboratory Supply/Equipment</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="N5" t="n">
-        <v>18</v>
-      </c>
-      <c r="O5" t="n">
-        <v>19</v>
-      </c>
-      <c r="P5" t="n">
         <v>5700</v>
       </c>
     </row>
@@ -744,57 +567,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.255204+00:00</t>
+          <t>INK CART, EPSON L3110, Black 003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>INK CART, EPSON L3110, Black 003</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
           <t>bottle</t>
         </is>
       </c>
+      <c r="D6" t="n">
+        <v>0.6899999999999999</v>
+      </c>
       <c r="E6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F6" t="n">
         <v>300</v>
       </c>
-      <c r="F6" t="n">
-        <v>25</v>
-      </c>
       <c r="G6" t="n">
-        <v>24</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>32</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PRINTER</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Office Supply</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="N6" t="n">
-        <v>18</v>
-      </c>
-      <c r="O6" t="n">
-        <v>24</v>
-      </c>
-      <c r="P6" t="n">
         <v>7200</v>
       </c>
     </row>
@@ -804,58 +594,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.556591+00:00</t>
+          <t>INK CART, EPSON L3110, Black 003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>INK CART, EPSON L3110, Black 003</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
           <t>bottle</t>
         </is>
       </c>
+      <c r="D7" t="n">
+        <v>0.6899999999999999</v>
+      </c>
       <c r="E7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" t="n">
         <v>300</v>
       </c>
-      <c r="F7" t="n">
-        <v>25</v>
-      </c>
       <c r="G7" t="n">
-        <v>25</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>32</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PRINTER</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Laboratory Supply/Equipment</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="N7" t="n">
-        <v>18</v>
-      </c>
-      <c r="O7" t="n">
-        <v>21</v>
-      </c>
-      <c r="P7" t="n">
-        <v>6300</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="8">
@@ -864,57 +621,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.255204+00:00</t>
+          <t>Toner Cart, Copier Muratec MFX - 2835 with ADF</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Toner Cart, Copier Muratec MFX - 2835 with ADF</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
           <t>cartridge</t>
         </is>
       </c>
+      <c r="D8" t="n">
+        <v>0.65</v>
+      </c>
       <c r="E8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" t="n">
         <v>3200</v>
       </c>
-      <c r="F8" t="n">
-        <v>8</v>
-      </c>
       <c r="G8" t="n">
-        <v>8</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>32</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PHOTOCOPYING MACHINE</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Office Supply</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" t="n">
-        <v>8</v>
-      </c>
-      <c r="P8" t="n">
         <v>25600</v>
       </c>
     </row>
@@ -924,174 +648,52 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.556591+00:00</t>
+          <t>Toner Cart, Copier Muratec MFX - 2835 with ADF</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Toner Cart, Copier Muratec MFX - 2835 with ADF</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
           <t>cartridge</t>
         </is>
       </c>
+      <c r="D9" t="n">
+        <v>0.65</v>
+      </c>
       <c r="E9" t="n">
+        <v>9</v>
+      </c>
+      <c r="F9" t="n">
         <v>3200</v>
       </c>
-      <c r="F9" t="n">
-        <v>9</v>
-      </c>
       <c r="G9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>32</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>INK/TONER FOR PHOTOCOPYING MACHINE</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Laboratory Supply/Equipment</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" t="n">
-        <v>6400</v>
+        <v>28800</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5303</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-27T16:12:37.255204+00:00</t>
+          <t>Unallocated Open Funds</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CLIP, backfold, 19mm, 12 pieces per box</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>box</t>
-        </is>
+          <t>PHP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.41</v>
       </c>
       <c r="E10" t="n">
-        <v>8.720000000000001</v>
+        <v>4498</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>32</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>COMMON OFFICE SUPPLIES</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Office Supply</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>1</v>
-      </c>
-      <c r="P10" t="n">
-        <v>8.720000000000001</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>5507</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-07-31T01:05:30.101366+00:00</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>aaa</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>aaa</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>32</v>
-      </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Office Supply</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" t="n">
-        <v>1</v>
+        <v>4498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>